<commit_message>
feat: add exceljs for data management
Install exceljs to enable Excel file operations and update index.html with caching headers and WebSocket error suppression.
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -417,310 +417,9 @@
     <col min="15" max="15" width="28.83203125" customWidth="1"/>
     <col min="16" max="16" width="22.83203125" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Category</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Scope</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Original Amount</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Original Currency</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Original Symbol</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Exchange Rate</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Total Amount</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Paid By</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Paid By ID</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Split Among</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Split Among IDs</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Split Type</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Notes</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Created Date</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>exp-1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2026-09-19</v>
-      </c>
-      <c r="C2" t="str">
-        <v>meal</v>
-      </c>
-      <c r="D2" t="str">
-        <v>shared</v>
-      </c>
-      <c r="E2">
-        <v>80</v>
-      </c>
-      <c r="F2" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="G2" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>80</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Ali</v>
-      </c>
-      <c r="K2" t="str">
-        <v>10002</v>
-      </c>
-      <c r="L2" t="str">
-        <v>HuiXin, Ali, Abu, Ahmad</v>
-      </c>
-      <c r="M2" t="str">
-        <v>10001,10002,10003,10004</v>
-      </c>
-      <c r="N2" t="str">
-        <v>equal</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-09-19T15:31:08.532Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>exp-2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-09-18</v>
-      </c>
-      <c r="C3" t="str">
-        <v>groceries</v>
-      </c>
-      <c r="D3" t="str">
-        <v>shared</v>
-      </c>
-      <c r="E3">
-        <v>48</v>
-      </c>
-      <c r="F3" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="G3" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>48</v>
-      </c>
-      <c r="J3" t="str">
-        <v>HuiXin</v>
-      </c>
-      <c r="K3" t="str">
-        <v>10001</v>
-      </c>
-      <c r="L3" t="str">
-        <v>HuiXin, Ali, Abu, Ahmad</v>
-      </c>
-      <c r="M3" t="str">
-        <v>10001,10002,10003,10004</v>
-      </c>
-      <c r="N3" t="str">
-        <v>equal</v>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v>2026-09-18T17:31:08.532Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>exp-3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-09-17</v>
-      </c>
-      <c r="C4" t="str">
-        <v>daily</v>
-      </c>
-      <c r="D4" t="str">
-        <v>shared</v>
-      </c>
-      <c r="E4">
-        <v>15</v>
-      </c>
-      <c r="F4" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="G4" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>15</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Abu</v>
-      </c>
-      <c r="K4" t="str">
-        <v>10003</v>
-      </c>
-      <c r="L4" t="str">
-        <v>HuiXin, Abu, Ahmad</v>
-      </c>
-      <c r="M4" t="str">
-        <v>10001,10003,10004</v>
-      </c>
-      <c r="N4" t="str">
-        <v>equal</v>
-      </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v>2026-09-17T17:31:08.532Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>exp-4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-09-16</v>
-      </c>
-      <c r="C5" t="str">
-        <v>transport</v>
-      </c>
-      <c r="D5" t="str">
-        <v>shared</v>
-      </c>
-      <c r="E5">
-        <v>24</v>
-      </c>
-      <c r="F5" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="G5" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>24</v>
-      </c>
-      <c r="J5" t="str">
-        <v>HuiXin</v>
-      </c>
-      <c r="K5" t="str">
-        <v>10001</v>
-      </c>
-      <c r="L5" t="str">
-        <v>HuiXin, Ali, Ahmad</v>
-      </c>
-      <c r="M5" t="str">
-        <v>10001,10002,10004</v>
-      </c>
-      <c r="N5" t="str">
-        <v>equal</v>
-      </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-      <c r="P5" t="str">
-        <v>2026-09-16T17:31:08.533Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>exp-5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-09-15</v>
-      </c>
-      <c r="C6" t="str">
-        <v>other</v>
-      </c>
-      <c r="D6" t="str">
-        <v>personal</v>
-      </c>
-      <c r="E6">
-        <v>28.5</v>
-      </c>
-      <c r="F6" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="G6" t="str">
-        <v>SGD</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>28.5</v>
-      </c>
-      <c r="J6" t="str">
-        <v>HuiXin</v>
-      </c>
-      <c r="K6" t="str">
-        <v>10001</v>
-      </c>
-      <c r="L6" t="str">
-        <v>HuiXin</v>
-      </c>
-      <c r="M6" t="str">
-        <v>10001</v>
-      </c>
-      <c r="N6" t="str">
-        <v>personal</v>
-      </c>
-      <c r="O6" t="str">
-        <v>Personal Study Books</v>
-      </c>
-      <c r="P6" t="str">
-        <v>2026-09-15T17:31:08.533Z</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>